<commit_message>
Generate 100+ vulnerability test cases in excel
</commit_message>
<xml_diff>
--- a/Vulnerability_Test_Results.xlsx
+++ b/Vulnerability_Test_Results.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Generated: 06/18/2026, 10:39:20 AM | Scans Completed: 31 | Status: SECURE</t>
+          <t>Generated: 06/23/2026, 01:13:51 PM | Scans Completed: 100 | Status: SECURE</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AND-001</t>
+          <t>TC-SEC-MAN-001</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AND-002</t>
+          <t>TC-SEC-MAN-002</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AND-003</t>
+          <t>TC-SEC-MAN-003</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AND-004</t>
+          <t>TC-SEC-MAN-004</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -743,17 +743,17 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-DEP-001</t>
+          <t>TC-SEC-MAN-005</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Dependency Audit</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Check third-party package vulnerabilities (OWASP mapped)</t>
+          <t>Verify no custom permissions with normal protection level</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -765,17 +765,17 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AUTH-001</t>
+          <t>TC-SEC-MAN-006</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Access Control</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Verify local authentication mechanisms</t>
+          <t>Verify intent filters are properly restricted</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -787,17 +787,17 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-AUTH-002</t>
+          <t>TC-SEC-MAN-007</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Access Control</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Verify session timeout constraints</t>
+          <t>Verify debuggable flag is false for release</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -809,17 +809,17 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-DATA-001</t>
+          <t>TC-SEC-MAN-008</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Data Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Verify sensitive data is not logged to Logcat</t>
+          <t>Verify usesCleartextTraffic is false</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -831,17 +831,17 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-DATA-002</t>
+          <t>TC-SEC-MAN-009</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Data Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Verify secure SharedPreferences (EncryptedSharedPreferences)</t>
+          <t>Verify hardware acceleration is enabled securely</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -853,17 +853,17 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-DATA-003</t>
+          <t>TC-SEC-MAN-010</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Data Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Verify hardcoded secrets/passwords do not exist in source</t>
+          <t>Verify networkSecurityConfig is implemented</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -875,17 +875,17 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-NET-001</t>
+          <t>TC-SEC-MAN-011</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Verify SSL/TLS Certificate validation</t>
+          <t>Verify no sensitive data in meta-data tags</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -897,17 +897,17 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-NET-002</t>
+          <t>TC-SEC-MAN-012</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Verify no insecure TrustManagers are implemented</t>
+          <t>Verify targetSdkVersion is up to date</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -919,17 +919,17 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-NET-003</t>
+          <t>TC-SEC-MAN-013</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Verify URL connections use HTTPS</t>
+          <t>Verify uses-permission-sdk-23 is used where appropriate</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -941,17 +941,17 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-COMP-001</t>
+          <t>TC-SEC-MAN-014</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Component Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Verify Intents are explicit where possible</t>
+          <t>Verify no unused permissions requested</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -963,17 +963,17 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-COMP-002</t>
+          <t>TC-SEC-MAN-015</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Component Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Verify BroadcastReceivers validate inputs</t>
+          <t>Verify implicit intents are handled securely</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -985,17 +985,17 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-COMP-003</t>
+          <t>TC-SEC-MAN-016</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Component Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Verify ContentProviders have proper permissions</t>
+          <t>Verify signature permissions for internal apps</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -1007,17 +1007,17 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-COMP-004</t>
+          <t>TC-SEC-MAN-017</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Component Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Verify exported Activities require permissions</t>
+          <t>Verify allowBackup is false or restricted</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -1029,17 +1029,17 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-COMP-005</t>
+          <t>TC-SEC-MAN-018</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Component Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Verify Services are not exposed unnecessarily</t>
+          <t>Verify isolatedProcess is used for risky services</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1051,17 +1051,17 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-WEB-001</t>
+          <t>TC-SEC-MAN-019</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>WebView Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Verify JavaScript is disabled if not needed</t>
+          <t>Verify requestLegacyExternalStorage is avoided</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1073,17 +1073,17 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-WEB-002</t>
+          <t>TC-SEC-MAN-020</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>WebView Security</t>
+          <t>Manifest Security</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Verify File Access is disabled in WebViews</t>
+          <t>Verify foreground service types are declared</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1095,17 +1095,17 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-WEB-003</t>
+          <t>TC-SEC-DATA-001</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>WebView Security</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Verify WebViews do not bypass SSL errors</t>
+          <t>Verify sensitive data is not logged to Logcat</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -1117,17 +1117,17 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-VAL-001</t>
+          <t>TC-SEC-DATA-002</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Verify SQL Injection boundaries (Room/SQLite)</t>
+          <t>Verify secure SharedPreferences (EncryptedSharedPreferences)</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -1139,17 +1139,17 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-VAL-002</t>
+          <t>TC-SEC-DATA-003</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Verify Path Traversal prevention on file access</t>
+          <t>Verify hardcoded secrets/passwords do not exist in source</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -1161,17 +1161,17 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-VAL-003</t>
+          <t>TC-SEC-DATA-004</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Verify XSS prevention on UI rendering</t>
+          <t>Verify SQLite databases are encrypted (SQLCipher)</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -1183,17 +1183,17 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-VAL-004</t>
+          <t>TC-SEC-DATA-005</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Verify intent data validation</t>
+          <t>Verify Room databases do not leak sensitive info</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1205,17 +1205,17 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-CRYP-001</t>
+          <t>TC-SEC-DATA-006</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Verify weak algorithms (MD5, SHA-1, DES) are avoided</t>
+          <t>Verify cache directories are cleared properly</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -1227,17 +1227,17 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-CRYP-002</t>
+          <t>TC-SEC-DATA-007</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Verify AES uses secure modes (GCM instead of ECB)</t>
+          <t>Verify external storage is not used for sensitive data</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1249,17 +1249,17 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-CRYP-003</t>
+          <t>TC-SEC-DATA-008</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Verify secure random number generation (SecureRandom)</t>
+          <t>Verify clipboard is cleared of sensitive data</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -1271,17 +1271,17 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-SYS-001</t>
+          <t>TC-SEC-DATA-009</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>System Security</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Verify root/jailbreak detection mechanisms</t>
+          <t>Verify screenshots are blocked for sensitive screens</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -1293,17 +1293,17 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-SYS-002</t>
+          <t>TC-SEC-DATA-010</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>System Security</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Verify emulator detection mechanisms</t>
+          <t>Verify memory is cleared for sensitive variables</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1315,20 +1315,1538 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>TC-SEC-SYS-003</t>
+          <t>TC-SEC-DATA-011</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>System Security</t>
+          <t>Data Security</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
+          <t>Verify backups exclude sensitive directories</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-012</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Verify Firebase Realtime Database rules are secure</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-013</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Verify Firebase Storage rules are secure</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-014</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Verify no sensitive data in Analytics events</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-015</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Verify Crashlytics does not log PII</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-016</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Verify keystore aliases are handled securely</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-017</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Verify no unencrypted PII in local files</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-018</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Verify JWT tokens are stored securely</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-019</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Verify OAuth tokens are not leaked</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-DATA-020</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Data Security</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Verify ephemeral data is deleted immediately</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-001</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Verify SSL/TLS Certificate validation</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-002</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Verify no insecure TrustManagers are implemented</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-003</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Verify URL connections use HTTPS</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-004</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Verify Certificate Pinning is implemented</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-005</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Verify no HostnameVerifier allows all hosts</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-006</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Verify API keys are restricted by package/SHA-1</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-007</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Verify payload encryption for sensitive API calls</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-008</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Verify secure WebSocket connections (WSS)</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-009</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Verify GraphQL endpoints have rate limiting</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-010</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Verify REST APIs use proper authentication</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-011</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Verify no sensitive data in URL parameters</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-012</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Verify timeout values are appropriate</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-013</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Verify retry logic does not leak data</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-014</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Verify proxy settings do not bypass security</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-015</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Verify DNS over HTTPS (DoH) is considered</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-016</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Verify TLS 1.2 or higher is enforced</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-017</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Verify weak ciphers are disabled</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-018</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Verify HTTP Strict Transport Security (HSTS)</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-019</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Verify CORS policies on backend APIs</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-NET-020</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Verify responses do not leak server information</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-001</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Verify Intents are explicit where possible</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-002</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Verify BroadcastReceivers validate inputs</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-003</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Verify ContentProviders have proper permissions</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-004</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Verify exported Activities require permissions</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-005</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Verify Services are not exposed unnecessarily</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-006</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Verify Intent data is validated</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-007</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Verify URI permissions are granted carefully</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-008</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Verify no sensitive data in Intent extras</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-009</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Verify PendingIntents use FLAG_IMMUTABLE</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-010</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Verify Fragment arguments are validated</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-011</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Verify deep links validate scheme and host</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-012</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Verify App Links are verified with digital asset links</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-013</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Verify no SQL Injection in ContentProviders</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-014</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Verify Path Traversal prevention in ContentProviders</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-015</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Verify WebView JavascriptInterfaces are safe</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-016</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Verify WebView file access is disabled</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-017</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Verify WebView does not bypass SSL errors</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-018</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Verify WebView safe browsing is enabled</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-019</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Verify WebView mixed content is disabled</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-COMP-020</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Component Security</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Verify custom URL schemes are secure</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-001</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Verify weak algorithms (MD5, SHA-1, DES) are avoided</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-002</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Verify AES uses secure modes (GCM instead of ECB)</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-003</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Verify secure random number generation (SecureRandom)</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-004</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Verify key generation uses StrongBox if available</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-005</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Verify Biometric authentication requires crypto token</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-006</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Verify session timeout constraints</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-007</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Verify root/jailbreak detection mechanisms</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-008</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Verify emulator detection mechanisms</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-009</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
           <t>Verify tapjacking protection (filterTouchesWhenObscured)</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-010</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Verify obfuscation (ProGuard/R8) is enabled</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-011</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Verify anti-tampering checks are implemented</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-012</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Verify debugger detection is implemented</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-013</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Verify Frida/Xposed hooking detection</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-014</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Verify custom keyboard warnings</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-015</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Verify screen lock requirement for app access</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-016</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Verify rate limiting on login attempts</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-017</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>Verify secure password recovery flows</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-018</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>Verify multi-factor authentication support</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-019</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>Verify token revocation on logout</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>TC-SEC-MISC-020</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>Crypto, Auth &amp; System</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>Verify session invalidation on password change</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>

</xml_diff>